<commit_message>
scan: seg8 2026-08-05 18:38 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-08-05.xlsx
+++ b/output/full_scan/batch_seq0_2026-08-05.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O116"/>
+  <dimension ref="A1:O117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4343,21 +4343,21 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>8105</v>
+        <v>8291</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>凌巨</t>
+          <t>尚茂</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>242.6700018244846</v>
+        <v>242.6927050273772</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>16.7</v>
+        <v>37.3</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.2868683110617</v>
+        <v>46.75365372686295</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>30.33857346329489</v>
+        <v>18.5689328585419</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.5544266683121233</v>
+        <v>0.4314013692969101</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.0107669101296838</v>
+        <v>0.7209759705218803</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>8213</v>
+        <v>8105</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>志超</t>
+          <t>凌巨</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>240.7224118185912</v>
+        <v>242.6700018244846</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>30.2</v>
+        <v>16.7</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>37.85705737106046</v>
+        <v>44.2868683110617</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>35.00455073798269</v>
+        <v>30.33857346329489</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.4784497442966357</v>
+        <v>0.5544266683121233</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.0279435734470043</v>
+        <v>-0.0107669101296838</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>8454</v>
+        <v>8213</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>富邦媒</t>
+          <t>志超</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>236.4399107209105</v>
+        <v>240.7224118185912</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>261.5</v>
+        <v>30.2</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>49.78816450040578</v>
+        <v>37.85705737106046</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>14.37842423480464</v>
+        <v>35.00455073798269</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>1.234495676617161</v>
+        <v>0.4784497442966357</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>2.033642267067881</v>
+        <v>-0.0279435734470043</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>8442</v>
+        <v>8454</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>威宏-KY</t>
+          <t>富邦媒</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>230.8510722991456</v>
+        <v>236.4399107209105</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>44.15</v>
+        <v>261.5</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>50.36781050417198</v>
+        <v>49.78816450040578</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>30.10189111247706</v>
+        <v>14.37842423480464</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.4985244347738281</v>
+        <v>1.234495676617161</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.2273919537206269</v>
+        <v>2.033642267067881</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>8499</v>
+        <v>8442</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>鼎炫-KY</t>
+          <t>威宏-KY</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>229.5559438270662</v>
+        <v>230.8510722991456</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>254</v>
+        <v>44.15</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>42.75211954866805</v>
+        <v>50.36781050417198</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>25.76571490476396</v>
+        <v>30.10189111247706</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.5670252403607693</v>
+        <v>0.4985244347738281</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-1.578387202566965</v>
+        <v>-0.2273919537206269</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4608,21 +4608,21 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>8390</v>
+        <v>8499</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>金益鼎</t>
+          <t>鼎炫-KY</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>226.9370715251494</v>
+        <v>229.5559438270662</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>95.3</v>
+        <v>254</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>45.03606806352831</v>
+        <v>42.75211954866805</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>35.10728547948727</v>
+        <v>25.76571490476396</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.7157273238843171</v>
+        <v>0.5670252403607693</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.5453421574450878</v>
+        <v>-1.578387202566965</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>8466</v>
+        <v>8390</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>金益鼎</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>225.6779149117172</v>
+        <v>226.9370715251494</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>16.85</v>
+        <v>95.3</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>49.59539262012203</v>
+        <v>45.03606806352831</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>20.52005503264594</v>
+        <v>35.10728547948727</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.2176602026973106</v>
+        <v>0.7157273238843171</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.0938921180048959</v>
+        <v>0.5453421574450878</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>8215</v>
+        <v>8466</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>明基材</t>
+          <t>美吉吉-KY</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>225.1785112073762</v>
+        <v>225.6779149117172</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>23.85</v>
+        <v>16.85</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>41.74702101470606</v>
+        <v>49.59539262012203</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>33.22319456121275</v>
+        <v>20.52005503264594</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.6305575255069015</v>
+        <v>0.2176602026973106</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.0107102290082095</v>
+        <v>-0.0938921180048959</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>9110</v>
+        <v>8215</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>越南控-DR</t>
+          <t>明基材</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>222.2511671150187</v>
+        <v>225.1785112073762</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>3.3</v>
+        <v>23.85</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>52.0346817392557</v>
+        <v>41.74702101470606</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>8.138199749885025</v>
+        <v>33.22319456121275</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.39622641509434</v>
+        <v>0.6305575255069015</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.0500572830201349</v>
+        <v>-0.0107102290082095</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, hist_turn_positive, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>8049</v>
+        <v>9110</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>晶采</t>
+          <t>越南控-DR</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>221.693543720159</v>
+        <v>222.2511671150187</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>26.3</v>
+        <v>3.3</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>51.68781196263362</v>
+        <v>52.0346817392557</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>14.06134527637303</v>
+        <v>8.138199749885025</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.559733431585023</v>
+        <v>1.39622641509434</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0622488140521292</v>
+        <v>0.0500572830201349</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
+          <t>macd_golden_cross, market_above_ma60, hist_turn_positive, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>8431</v>
+        <v>8049</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>匯鑽科</t>
+          <t>晶采</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>218.1029980511149</v>
+        <v>221.693543720159</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>50.9</v>
+        <v>26.3</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>54.13426474190627</v>
+        <v>51.68781196263362</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>19.02121114250714</v>
+        <v>14.06134527637303</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1.536357395574801</v>
+        <v>0.559733431585023</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.5780824512718916</v>
+        <v>0.0622488140521292</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>8076</v>
+        <v>8431</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>伍豐</t>
+          <t>匯鑽科</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>215.7956530566229</v>
+        <v>218.1029980511149</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>23.3</v>
+        <v>50.9</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>45.8129983338923</v>
+        <v>54.13426474190627</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>14.24518017642697</v>
+        <v>19.02121114250714</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.6706422976001176</v>
+        <v>1.536357395574801</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.0129062852494695</v>
+        <v>0.5780824512718916</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>volume_break, market_above_ma60, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>8481</v>
+        <v>8076</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>政伸</t>
+          <t>伍豐</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>211.7113109889153</v>
+        <v>215.7956530566229</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>40</v>
+        <v>23.3</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,16 +5004,16 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>39.31710890441436</v>
+        <v>45.8129983338923</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>22.37378607597904</v>
+        <v>14.24518017642697</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.2354756304221362</v>
+        <v>0.6706422976001176</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.09497485205618079</v>
+        <v>-0.0129062852494695</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>8487</v>
+        <v>8481</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>愛爾達-創</t>
+          <t>政伸</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>209.7700576360122</v>
+        <v>211.7113109889153</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>74.90000000000001</v>
+        <v>40</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>40.16380582127694</v>
+        <v>39.31710890441436</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>16.39894379894718</v>
+        <v>22.37378607597904</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.7043862309995544</v>
+        <v>0.2354756304221362</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.0659479462557772</v>
+        <v>-0.09497485205618079</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>9105</v>
+        <v>8487</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>泰金寶-DR</t>
+          <t>愛爾達-創</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>208.2413830315833</v>
+        <v>209.7700576360122</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>8.210000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>45.68854990393852</v>
+        <v>40.16380582127694</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>19.26675434574226</v>
+        <v>16.39894379894718</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.8675808882145409</v>
+        <v>0.7043862309995544</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.0115385656145282</v>
+        <v>0.0659479462557772</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>8162</v>
+        <v>9105</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>微矽電子-創</t>
+          <t>泰金寶-DR</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>205.6378019027187</v>
+        <v>208.2413830315833</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>52.5</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>37.17306344091449</v>
+        <v>45.68854990393852</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>36.2227029620643</v>
+        <v>19.26675434574226</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.6148196874915759</v>
+        <v>0.8675808882145409</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-1.010772359363811</v>
+        <v>-0.0115385656145282</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>8240</v>
+        <v>8162</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>華宏</t>
+          <t>微矽電子-創</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>205.3060424359474</v>
+        <v>205.6378019027187</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>41.75</v>
+        <v>52.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>40.75851713367297</v>
+        <v>37.17306344091449</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>41.78115924949694</v>
+        <v>36.2227029620643</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.8252688155895923</v>
+        <v>0.6148196874915759</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.4473977706434286</v>
+        <v>-1.010772359363811</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>8422</v>
+        <v>8240</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>可寧衛*</t>
+          <t>華宏</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>203.9058810441245</v>
+        <v>205.3060424359474</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>26</v>
+        <v>41.75</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>47.50073782212741</v>
+        <v>40.75851713367297</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>15.67394214571042</v>
+        <v>41.78115924949694</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.5991816743091029</v>
+        <v>0.8252688155895923</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.09859850767117299</v>
+        <v>0.4473977706434286</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>8091</v>
+        <v>8422</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>翔名</t>
+          <t>可寧衛*</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>193.8488504929947</v>
+        <v>203.9058810441245</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>229</v>
+        <v>26</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,16 +5322,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>45.24800020268185</v>
+        <v>47.50073782212741</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>19.04087308864152</v>
+        <v>15.67394214571042</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4899470605129356</v>
+        <v>0.5991816743091029</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.902307025881175</v>
+        <v>0.09859850767117299</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>8131</v>
+        <v>8091</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>福懋科</t>
+          <t>翔名</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>188.8483707807493</v>
+        <v>193.8488504929947</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>66</v>
+        <v>229</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,16 +5375,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>49.35205558413239</v>
+        <v>45.24800020268185</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>16.0409079889905</v>
+        <v>19.04087308864152</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1.061667949964766</v>
+        <v>0.4899470605129356</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.240020607784261</v>
+        <v>-2.902307025881175</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5403,21 +5403,21 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>8092</v>
+        <v>8131</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>建暐</t>
+          <t>福懋科</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>185.8422717287602</v>
+        <v>188.8483707807493</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>13.45</v>
+        <v>66</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>44.85684810583544</v>
+        <v>49.35205558413239</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>15.39869706375627</v>
+        <v>16.0409079889905</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.4010818114945469</v>
+        <v>1.061667949964766</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0536438964913277</v>
+        <v>-0.240020607784261</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>8455</v>
+        <v>8092</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>大拓-KY</t>
+          <t>建暐</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>177.9068082908403</v>
+        <v>185.8422717287601</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>23.95</v>
+        <v>13.45</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>40.82751151425108</v>
+        <v>44.85684810583544</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>18.11612844099954</v>
+        <v>15.39869706375627</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.9574693720899696</v>
+        <v>0.4010818114945469</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0267872999702787</v>
+        <v>0.0536438964913277</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>8467</v>
+        <v>8455</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>波力-KY</t>
+          <t>大拓-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>171.539772218706</v>
+        <v>177.9068082908403</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>98.5</v>
+        <v>23.95</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>39.22952858218727</v>
+        <v>40.82751151425108</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>15.80674436429138</v>
+        <v>18.11612844099954</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.6418179423148607</v>
+        <v>0.9574693720899696</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0604539490037554</v>
+        <v>0.0267872999702787</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>8104</v>
+        <v>8467</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>錸寶</t>
+          <t>波力-KY</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>171.3953345102688</v>
+        <v>171.539772218706</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>31.2</v>
+        <v>98.5</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>38.80481182803485</v>
+        <v>39.22952858218727</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>31.41652466603397</v>
+        <v>15.80674436429138</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3450932987406983</v>
+        <v>0.6418179423148607</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.2569022944030319</v>
+        <v>0.0604539490037554</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>8183</v>
+        <v>8104</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>精星</t>
+          <t>錸寶</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>171.3420872692566</v>
+        <v>171.3953345102688</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>29.35</v>
+        <v>31.2</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>41.72109606876234</v>
+        <v>38.80481182803485</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>27.33559472855245</v>
+        <v>31.41652466603397</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.4015579956822988</v>
+        <v>0.3450932987406983</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.1333839322891039</v>
+        <v>-0.2569022944030319</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8477</v>
+        <v>8183</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>創業家</t>
+          <t>精星</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>167.4254417972556</v>
+        <v>171.3420872692566</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>15.9</v>
+        <v>29.35</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>51.42739279343411</v>
+        <v>41.72109606876234</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>10.35894276825896</v>
+        <v>27.33559472855245</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.9593470737124852</v>
+        <v>0.4015579956822988</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.3242589247812351</v>
+        <v>-0.1333839322891039</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8085</v>
+        <v>8477</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>福華</t>
+          <t>創業家</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>165.3937346717612</v>
+        <v>167.4254417972556</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>11.15</v>
+        <v>15.9</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>43.53335223315796</v>
+        <v>51.42739279343411</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>15.31063077688704</v>
+        <v>10.35894276825896</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>3.145587872612502</v>
+        <v>0.9593470737124852</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.0168073699512702</v>
+        <v>0.3242589247812351</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>8404</v>
+        <v>8085</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>百和興業-KY</t>
+          <t>福華</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>164.4923930646651</v>
+        <v>165.3937346717612</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>16.2</v>
+        <v>11.15</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>39.00637360893367</v>
+        <v>43.53335223315796</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>18.493805136096</v>
+        <v>15.31063077688704</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.4841200953670905</v>
+        <v>3.145587872612502</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0547131227077339</v>
+        <v>0.0168073699512702</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>8410</v>
+        <v>8404</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>森田</t>
+          <t>百和興業-KY</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>161.9685441204396</v>
+        <v>164.4923930646651</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>30.9</v>
+        <v>16.2</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>40.25399775456486</v>
+        <v>39.00637360893367</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>30.57203129466938</v>
+        <v>18.493805136096</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.6485618141770624</v>
+        <v>0.4841200953670905</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0352822420871223</v>
+        <v>-0.0547131227077339</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>8089</v>
+        <v>8410</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>康全電訊</t>
+          <t>森田</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>161.1977815258585</v>
+        <v>161.9685441204396</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>18.35</v>
+        <v>30.9</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>43.14020031862088</v>
+        <v>40.25399775456486</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>15.7304289952431</v>
+        <v>30.57203129466938</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.3930862234716922</v>
+        <v>0.6485618141770624</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0482599307594878</v>
+        <v>-0.0352822420871223</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>8463</v>
+        <v>8089</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>潤泰材</t>
+          <t>康全電訊</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>158.354911391203</v>
+        <v>161.1977815258585</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>20.95</v>
+        <v>18.35</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>40.90038711689992</v>
+        <v>43.14020031862088</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>20.5074606028912</v>
+        <v>15.7304289952431</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.8735343964552327</v>
+        <v>0.3930862234716922</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.0287864368458514</v>
+        <v>-0.0482599307594878</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>8171</v>
+        <v>8463</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>天宇</t>
+          <t>潤泰材</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>157.3664786797888</v>
+        <v>158.354911391203</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>19.5</v>
+        <v>20.95</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>39.44729213373165</v>
+        <v>40.90038711689992</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.45005059461626</v>
+        <v>20.5074606028912</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.7448831390526537</v>
+        <v>0.8735343964552327</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0228060227340787</v>
+        <v>-0.0287864368458514</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8341</v>
+        <v>8171</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>日友</t>
+          <t>天宇</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>147.8310732182628</v>
+        <v>157.3664786797888</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>75.3</v>
+        <v>19.5</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>42.56493336150044</v>
+        <v>39.44729213373165</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>13.06496744477233</v>
+        <v>15.45005059461626</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.4864092257367006</v>
+        <v>0.7448831390526537</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0667978227483523</v>
+        <v>-0.0228060227340787</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>9902</v>
+        <v>8341</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>台火</t>
+          <t>日友</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>144.3145012602367</v>
+        <v>147.8310732182628</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>13.7</v>
+        <v>75.3</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>49.48352210560945</v>
+        <v>42.56493336150044</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>8.61929380723007</v>
+        <v>13.06496744477233</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.886385711270161</v>
+        <v>0.4864092257367006</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.0047672132924186</v>
+        <v>-0.0667978227483523</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6145,21 +6145,21 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>9906</v>
+        <v>9902</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>欣巴巴</t>
+          <t>台火</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>140.3996038461496</v>
+        <v>144.3145012602367</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>39.4</v>
+        <v>13.7</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>45.84453571083127</v>
+        <v>49.48352210560945</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>12.27135729134538</v>
+        <v>8.61929380723007</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.3444355689874573</v>
+        <v>0.886385711270161</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.1179622716808762</v>
+        <v>0.0047672132924186</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>8940</v>
+        <v>9906</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>新天地</t>
+          <t>欣巴巴</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>138.9531188298891</v>
+        <v>140.3996038461496</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>15.35</v>
+        <v>39.4</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>26.00917195145058</v>
+        <v>45.84453571083127</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15.71496843155526</v>
+        <v>12.27135729134538</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.6197446962138639</v>
+        <v>0.3444355689874573</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.0593695358770107</v>
+        <v>-0.1179622716808762</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8478</v>
+        <v>8940</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>東哥遊艇</t>
+          <t>新天地</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>136.6751594024192</v>
+        <v>138.9531188298891</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>150.5</v>
+        <v>15.35</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>45.86283952051385</v>
+        <v>26.00917195145058</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>8.507534092477634</v>
+        <v>15.71496843155526</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.8093088292213524</v>
+        <v>0.6197446962138639</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0340487813131498</v>
+        <v>-0.0593695358770107</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>8472</v>
+        <v>8478</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>夠麻吉</t>
+          <t>東哥遊艇</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>130.3374108904015</v>
+        <v>136.6751594024192</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>68.2</v>
+        <v>150.5</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>34.68331776014529</v>
+        <v>45.86283952051385</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.32870414095225</v>
+        <v>8.507534092477634</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4807881773399015</v>
+        <v>0.8093088292213524</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.2953421339722908</v>
+        <v>-0.0340487813131498</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>8084</v>
+        <v>8472</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>巨虹</t>
+          <t>夠麻吉</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>125.0616571829062</v>
+        <v>130.3374108904015</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>41.85</v>
+        <v>68.2</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>38.89463693235169</v>
+        <v>34.68331776014529</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>18.49061565829323</v>
+        <v>17.32870414095225</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.2114780107824544</v>
+        <v>0.4807881773399015</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1958930323713181</v>
+        <v>-0.2953421339722908</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>8482</v>
+        <v>8084</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>商億-KY</t>
+          <t>巨虹</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>124.2047096209879</v>
+        <v>125.0616571829062</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0</v>
+        <v>41.85</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>26.65841941489174</v>
+        <v>38.89463693235169</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>6.729856451837642</v>
+        <v>18.49061565829323</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.0037714975359549</v>
+        <v>0.2114780107824544</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-3.308761445058688</v>
+        <v>-0.1958930323713181</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>9136</v>
+        <v>8482</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>巨騰-DR</t>
+          <t>商億-KY</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>93.5725803003636</v>
+        <v>124.2047096209879</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.98497103629405</v>
+        <v>26.65841941489174</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>15.68666088621908</v>
+        <v>6.729856451837642</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.6938623155297506</v>
+        <v>0.0037714975359549</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.0016104579426809</v>
+        <v>-3.308761445058688</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>8176</v>
+        <v>9136</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>智捷</t>
+          <t>巨騰-DR</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>57.28474810738341</v>
+        <v>93.5725803003636</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>9.92</v>
+        <v>11.35</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>46.50302599544024</v>
+        <v>42.98497103629405</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>11.09024144819485</v>
+        <v>15.68666088621908</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.8193074864267864</v>
+        <v>0.6938623155297506</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,62 +6559,115 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0066239968344047</v>
+        <v>-0.0016104579426809</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
+        <v>8176</v>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>智捷</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>57.28474810738341</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>46.50302599544024</v>
+      </c>
+      <c r="I116" s="2" t="n">
+        <v>11.09024144819485</v>
+      </c>
+      <c r="J116" s="2" t="n">
+        <v>0.8193074864267864</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N116" s="2" t="n">
+        <v>-0.0066239968344047</v>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
         <v>8277</v>
       </c>
-      <c r="B116" s="2" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>商丞</t>
         </is>
       </c>
-      <c r="C116" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D116" s="2" t="n">
+      <c r="C117" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D117" s="2" t="n">
         <v>19.92036312274531</v>
       </c>
-      <c r="E116" s="2" t="n">
+      <c r="E117" s="2" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H116" s="2" t="n">
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H117" s="2" t="n">
         <v>45.7098484518366</v>
       </c>
-      <c r="I116" s="2" t="n">
+      <c r="I117" s="2" t="n">
         <v>19.10433902193053</v>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J117" s="2" t="n">
         <v>0.5207919761533887</v>
       </c>
-      <c r="K116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M116" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N116" s="2" t="n">
+      <c r="K117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N117" s="2" t="n">
         <v>0.05087062687089</v>
       </c>
-      <c r="O116" s="2" t="inlineStr">
+      <c r="O117" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60</t>
         </is>

</xml_diff>